<commit_message>
Chart color change and bug fix.
</commit_message>
<xml_diff>
--- a/data/Goal_Habit_Tracker_2026_2027.xlsx
+++ b/data/Goal_Habit_Tracker_2026_2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shuvadeep\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shuvadeep\Documents\habit_tracker_app_fixed\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{556F3998-425D-4877-8B33-F2AED466C09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12550A2D-D148-4A71-968F-A743DA10DB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="131">
   <si>
     <t>24-Month Goal &amp; Habit Dashboard</t>
   </si>
@@ -432,6 +432,9 @@
   <si>
     <t>De-Motivated</t>
   </si>
+  <si>
+    <t>Best Day</t>
+  </si>
 </sst>
 </file>
 
@@ -808,10 +811,10 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0.79545454545454541</c:v>
+                  <c:v>0.75757575757575746</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.79545454545454541</c:v>
+                  <c:v>0.74675324675324672</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1825,7 +1828,7 @@
       </c>
       <c r="B3" s="3">
         <f>IFERROR(AVERAGE('Daily Tracker'!N2:N366),"")</f>
-        <v>0.79545454545454541</v>
+        <v>0.75757575757575746</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1834,7 +1837,7 @@
       </c>
       <c r="B4" s="3">
         <f>IFERROR(AVERAGE('Weekly Review'!I2:I53),"")</f>
-        <v>0.79545454545454541</v>
+        <v>0.74675324675324672</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -2173,20 +2176,42 @@
       <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="3" t="str">
+      <c r="C6" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="N6" s="3">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.81818181818181823</v>
       </c>
       <c r="O6" s="2"/>
     </row>
@@ -2197,20 +2222,42 @@
       <c r="B7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="3" t="str">
+      <c r="C7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="N7" s="3">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.81818181818181823</v>
       </c>
       <c r="O7" s="2"/>
     </row>
@@ -2221,20 +2268,42 @@
       <c r="B8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="3" t="str">
+      <c r="C8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="N8" s="3">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.54545454545454541</v>
       </c>
       <c r="O8" s="2"/>
     </row>
@@ -2245,20 +2314,42 @@
       <c r="B9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="3" t="str">
+      <c r="C9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="N9" s="3">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.45454545454545453</v>
       </c>
       <c r="O9" s="2"/>
     </row>
@@ -2269,22 +2360,46 @@
       <c r="B10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="3" t="str">
+      <c r="C10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="N10" s="3">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="O10" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
@@ -10916,28 +11031,28 @@
       </c>
       <c r="C2" s="2">
         <f>COUNTIF('Daily Tracker'!C2:C8,"✓")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="2">
         <f>COUNTIF('Daily Tracker'!D2:D8,"✓")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" s="2">
         <f>COUNTIF('Daily Tracker'!E2:E8,"✓")</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F2" s="2">
         <f>COUNTIF('Daily Tracker'!G2:G8,"✓")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3">
         <f>IFERROR(AVERAGE('Daily Tracker'!N2:N8),"")</f>
-        <v>0.79545454545454541</v>
+        <v>0.76623376623376616</v>
       </c>
       <c r="I2" s="3">
         <f t="shared" ref="I2:I33" si="0">IF(H2="","",H2)</f>
-        <v>0.79545454545454541</v>
+        <v>0.76623376623376616</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -10952,28 +11067,28 @@
       </c>
       <c r="C3" s="2">
         <f>COUNTIF('Daily Tracker'!C9:C15,"✓")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2">
         <f>COUNTIF('Daily Tracker'!D9:D15,"✓")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2">
         <f>COUNTIF('Daily Tracker'!E9:E15,"✓")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="2">
         <f>COUNTIF('Daily Tracker'!G9:G15,"✓")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="3" t="str">
+      <c r="H3" s="3">
         <f>IFERROR(AVERAGE('Daily Tracker'!N9:N15),"")</f>
-        <v/>
-      </c>
-      <c r="I3" s="3" t="str">
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="I3" s="3">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.72727272727272729</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>

</xml_diff>